<commit_message>
thêm preview khóa học trong trang phê duyệt khóa học
</commit_message>
<xml_diff>
--- a/src/main/resources/database/danh_sach_lop.xlsx
+++ b/src/main/resources/database/danh_sach_lop.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29214"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29216"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thanh\OneDrive\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ADDBB4E7-8BCB-4BD9-A1EA-6A80BCAACA05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63F99D52-0269-4C2F-BAE1-A0698DA6A699}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="67">
   <si>
     <t>STT</t>
   </si>
@@ -212,6 +212,15 @@
   </si>
   <si>
     <t>0847483176</t>
+  </si>
+  <si>
+    <t>Jane Student</t>
+  </si>
+  <si>
+    <t>jane@student.com</t>
+  </si>
+  <si>
+    <t>0903456789</t>
   </si>
 </sst>
 </file>
@@ -356,8 +365,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{304543A8-35CD-4643-BFB1-C8EE96027DE1}" name="Table1" displayName="Table1" ref="A1:D21" totalsRowShown="0" headerRowDxfId="7" dataDxfId="5" headerRowBorderDxfId="6" tableBorderDxfId="4">
-  <autoFilter ref="A1:D21" xr:uid="{304543A8-35CD-4643-BFB1-C8EE96027DE1}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{304543A8-35CD-4643-BFB1-C8EE96027DE1}" name="Table1" displayName="Table1" ref="A1:D22" totalsRowShown="0" headerRowDxfId="7" dataDxfId="5" headerRowBorderDxfId="6" tableBorderDxfId="4">
+  <autoFilter ref="A1:D22" xr:uid="{304543A8-35CD-4643-BFB1-C8EE96027DE1}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{883621F8-ABAE-418C-9654-5C3970356BDB}" name="STT" dataDxfId="3"/>
     <tableColumn id="2" xr3:uid="{F4263740-121D-42C8-9DC4-685D56FA24E7}" name="Họ tên" dataDxfId="2"/>
@@ -655,7 +664,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D21"/>
+  <dimension ref="A1:D22"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="9" style="2"/>
@@ -684,13 +693,13 @@
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>4</v>
+        <v>64</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>24</v>
+        <v>65</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>44</v>
+        <v>66</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.2">
@@ -698,13 +707,13 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
@@ -712,13 +721,13 @@
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
@@ -726,13 +735,13 @@
         <v>4</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.2">
@@ -740,13 +749,13 @@
         <v>5</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.2">
@@ -754,13 +763,13 @@
         <v>6</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.2">
@@ -768,13 +777,13 @@
         <v>7</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.2">
@@ -782,13 +791,13 @@
         <v>8</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.2">
@@ -796,13 +805,13 @@
         <v>9</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.2">
@@ -810,13 +819,13 @@
         <v>10</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.2">
@@ -824,13 +833,13 @@
         <v>11</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.2">
@@ -838,13 +847,13 @@
         <v>12</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.2">
@@ -852,13 +861,13 @@
         <v>13</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.2">
@@ -866,13 +875,13 @@
         <v>14</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.2">
@@ -880,13 +889,13 @@
         <v>15</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.2">
@@ -894,13 +903,13 @@
         <v>16</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.2">
@@ -908,13 +917,13 @@
         <v>17</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.2">
@@ -922,13 +931,13 @@
         <v>18</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.2">
@@ -936,13 +945,13 @@
         <v>19</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.2">
@@ -950,12 +959,26 @@
         <v>20</v>
       </c>
       <c r="B21" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A22" s="2">
+        <v>21</v>
+      </c>
+      <c r="B22" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="C21" s="1" t="s">
+      <c r="C22" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="D21" s="1" t="s">
+      <c r="D22" s="1" t="s">
         <v>63</v>
       </c>
     </row>

</xml_diff>